<commit_message>
Fix DI tri-set A: swap cable fly exercises for equipment compatibility
Cable fly low-to-high moved to finisher (after barbell dismantled), butterfly cable from top moved into tri-set A (cable already high via spotter arms).

https://claude.ai/code/session_01GVJ1XP4t8b95djSt71eE5q
</commit_message>
<xml_diff>
--- a/fitness_plan_david_v3.xlsx
+++ b/fitness_plan_david_v3.xlsx
@@ -2321,6 +2321,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -2360,7 +2362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2705,7 +2707,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -2755,7 +2757,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3005,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -3047,7 +3049,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3092,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -3841,6 +3846,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -4604,6 +4611,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -5463,6 +5472,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -5502,7 +5513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5847,7 +5858,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -5897,7 +5908,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6156,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -6189,7 +6200,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6243,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -6983,6 +6997,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -7746,6 +7762,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -8605,6 +8623,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -8644,7 +8664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8989,7 +9009,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -9039,7 +9059,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -9287,7 +9307,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -9331,7 +9351,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9394,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -10841,6 +10864,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -11604,6 +11629,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -12463,6 +12490,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -12502,7 +12531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12847,7 +12876,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -12897,7 +12926,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -13145,7 +13174,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -13189,7 +13218,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -13232,7 +13261,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -13983,6 +14015,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -14746,6 +14780,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -15605,6 +15641,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -15644,7 +15682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -15989,7 +16027,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -16039,7 +16077,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -16287,7 +16325,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -16331,7 +16369,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -16374,7 +16412,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -17125,6 +17166,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -17888,6 +17931,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -17927,7 +17972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -18272,7 +18317,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -18322,7 +18367,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -18570,7 +18615,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -18614,7 +18659,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -18657,7 +18702,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -19516,6 +19564,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -19555,7 +19605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -19900,7 +19950,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -19950,7 +20000,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -20198,7 +20248,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -20242,7 +20292,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -20285,7 +20335,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -21036,6 +21089,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -21799,6 +21854,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -22658,6 +22715,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -23409,6 +23468,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -24172,6 +24233,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">
@@ -25031,6 +25094,8 @@
         </is>
       </c>
       <c r="J23" s="44" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -25070,7 +25135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -25415,7 +25480,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>Kabel Fly tief→hoch (Schrägbank)</t>
+          <t>Butterfly Kabelzug von oben</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
@@ -25465,7 +25530,7 @@
       <c r="T11" s="15" t="inlineStr"/>
       <c r="U11" s="37" t="inlineStr">
         <is>
-          <t>Kabel von unten, kreuzen oben</t>
+          <t>Kabel bereits oben — kein Umbau nötig</t>
         </is>
       </c>
     </row>
@@ -25713,7 +25778,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Butterfly Kabelzug von oben</t>
+          <t>Kabel Fly tief→hoch (Schrägbank)</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -25757,7 +25822,7 @@
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="37" t="inlineStr">
         <is>
-          <t>Brustkontraktion maximal</t>
+          <t>LH abgebaut → Kabel jetzt nach unten, Schrägbank</t>
         </is>
       </c>
     </row>
@@ -25800,7 +25865,10 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
-    </row>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -26551,6 +26619,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
@@ -27314,6 +27384,8 @@
         </is>
       </c>
       <c r="J21" s="44" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="48" t="inlineStr">

</xml_diff>

<commit_message>
Reduce leg day to 3 sets and replace Beinbeuger exercise
Cut 4th set on all SA (leg day) exercises from W3 onward due to repeated fatigue/abandoned sets. Replaced lying dumbbell leg curl (broken by missing equipment) with standing cable leg curl (ankle strap) until ordered leg-curl bench arrives. Updated technique sheet link accordingly.

https://claude.ai/code/session_01GVJ1XP4t8b95djSt71eE5q
</commit_message>
<xml_diff>
--- a/fitness_plan_david_v3.xlsx
+++ b/fitness_plan_david_v3.xlsx
@@ -395,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -603,6 +603,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -970,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K34"/>
+  <dimension ref="B2:K34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -2667,7 +2673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="B2:V23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -3400,7 +3406,6 @@
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="47" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="21.95" customHeight="1" s="33">
       <c r="B23" s="58" t="inlineStr">
         <is>
@@ -3439,7 +3444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="B2:V23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -4154,7 +4159,6 @@
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="47" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="21.95" customHeight="1" s="33">
       <c r="B23" s="58" t="inlineStr">
         <is>
@@ -4193,7 +4197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="B2:V23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -4312,11 +4316,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -4456,16 +4459,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -4516,16 +4513,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="74" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -4576,16 +4567,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -4665,16 +4650,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -4687,7 +4666,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -4731,7 +4710,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -4779,16 +4758,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>
@@ -4920,7 +4893,6 @@
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="47" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="21.95" customHeight="1" s="33">
       <c r="B23" s="35" t="inlineStr">
         <is>
@@ -4959,7 +4931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="B2:V25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -5782,7 +5754,6 @@
       <c r="K23" s="46" t="n"/>
       <c r="L23" s="47" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25" ht="21.95" customHeight="1" s="33">
       <c r="B25" s="58" t="inlineStr">
         <is>
@@ -7464,11 +7435,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -7608,16 +7578,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -7668,16 +7632,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -7728,16 +7686,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -7817,16 +7769,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -7839,7 +7785,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -7883,7 +7829,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -7931,16 +7877,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>
@@ -9742,7 +9682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E35"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="33" min="1" max="1"/>
@@ -10156,7 +10096,7 @@
       </c>
       <c r="C23" s="53" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -10166,7 +10106,7 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>▶  YouTube Tutorial öffnen →  Beinbeuger mit KH liegend</t>
+          <t>▶  YouTube Tutorial öffnen →  Stehender Kabel-Beinbeuger</t>
         </is>
       </c>
     </row>
@@ -11330,11 +11270,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -11474,16 +11413,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -11534,16 +11467,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -11594,16 +11521,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -11683,16 +11604,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -11705,7 +11620,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -11749,7 +11664,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -11797,16 +11712,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>
@@ -14480,11 +14389,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -14624,16 +14532,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -14684,16 +14586,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -14744,16 +14640,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -14833,16 +14723,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -14855,7 +14739,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -14899,7 +14783,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -14947,16 +14831,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>
@@ -17630,11 +17508,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -17774,16 +17651,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -17834,16 +17705,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -17894,16 +17759,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -17983,16 +17842,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -18005,7 +17858,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -18049,7 +17902,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -18097,16 +17950,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>
@@ -21665,11 +21512,10 @@
           <t>SATZ 3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
-        <is>
-          <t>SATZ 4</t>
-        </is>
-      </c>
+      <c r="Q6" s="75" t="inlineStr"/>
+      <c r="R6" s="46" t="n"/>
+      <c r="S6" s="46" t="n"/>
+      <c r="T6" s="47" t="n"/>
       <c r="U6" s="41" t="inlineStr">
         <is>
           <t>NOTIZEN</t>
@@ -21809,16 +21655,10 @@
       </c>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="R9" s="23" t="inlineStr">
-        <is>
-          <t>5–8</t>
-        </is>
-      </c>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
+      <c r="Q9" s="74" t="inlineStr"/>
+      <c r="R9" s="76" t="inlineStr"/>
+      <c r="S9" s="68" t="inlineStr"/>
+      <c r="T9" s="68" t="inlineStr"/>
       <c r="U9" s="24" t="inlineStr">
         <is>
           <t>Tiefe Kniebeuge, Fersen am Boden</t>
@@ -21869,16 +21709,10 @@
       </c>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="R10" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
+      <c r="Q10" s="74" t="inlineStr"/>
+      <c r="R10" s="76" t="inlineStr"/>
+      <c r="S10" s="68" t="inlineStr"/>
+      <c r="T10" s="68" t="inlineStr"/>
       <c r="U10" s="24" t="inlineStr">
         <is>
           <t>Hinteres Bein auf Bank, Knie 90°</t>
@@ -21929,16 +21763,10 @@
       </c>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
-      <c r="Q11" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R11" s="23" t="inlineStr">
-        <is>
-          <t>8–10</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
+      <c r="Q11" s="74" t="inlineStr"/>
+      <c r="R11" s="76" t="inlineStr"/>
+      <c r="S11" s="68" t="inlineStr"/>
+      <c r="T11" s="68" t="inlineStr"/>
       <c r="U11" s="24" t="inlineStr">
         <is>
           <t>Schultern auf Bank, Hüfte oben pressen</t>
@@ -22018,16 +21846,10 @@
       </c>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="22" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>6–8</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
+      <c r="Q14" s="74" t="inlineStr"/>
+      <c r="R14" s="76" t="inlineStr"/>
+      <c r="S14" s="68" t="inlineStr"/>
+      <c r="T14" s="68" t="inlineStr"/>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>Leichtes Kniebeugen, Rücken gerade</t>
@@ -22040,7 +21862,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Beinbeuger mit KH liegend</t>
+          <t>Stehender Kabel-Beinbeuger (Ankle Strap)</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -22084,7 +21906,7 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>KH zwischen Füße, langsam runter</t>
+          <t>Pro Bein, Ankle Strap am Kabelturm — Ersatz bis Leg-Trainer-Bank da ist</t>
         </is>
       </c>
     </row>
@@ -22132,16 +21954,10 @@
       </c>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="R16" s="23" t="inlineStr">
-        <is>
-          <t>10–12</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="Q16" s="74" t="inlineStr"/>
+      <c r="R16" s="76" t="inlineStr"/>
+      <c r="S16" s="68" t="inlineStr"/>
+      <c r="T16" s="68" t="inlineStr"/>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>Volle Bewegung, Pause oben 1 sek</t>

</xml_diff>